<commit_message>
Add Excel file for type aliases and number systems tests
</commit_message>
<xml_diff>
--- a/tests/01.csharp/13.network-programming/07.http-fundamentals.xlsx
+++ b/tests/01.csharp/13.network-programming/07.http-fundamentals.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,7 +476,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>До якого рівня мережевої моделі OSI відноситься протокол HTTP?</t>
+          <t>На якому рівні мережевої моделі OSI працює протокол HTTP?</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -486,44 +486,46 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Прикладний рівень (Application Layer, Layer 7)</t>
+          <t>Фізичний рівень (Layer 1)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Транспортний рівень (Transport Layer, Layer 4)</t>
+          <t>Транспортний рівень (Layer 4)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Мережевий рівень (Network Layer, Layer 3)</t>
+          <t>Мережевий рівень (Layer 3)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Фізичний рівень (Physical Layer, Layer 1)</t>
+          <t>Прикладний рівень (Layer 7)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>30</v>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>HTTP є протоколом прикладного рівня (Layer 7 моделі OSI). Він визначає семантику взаємодії між клієнтом і сервером, тоді як безпосередню доставку байтів здійснюють нижчі рівні (наприклад, TCP на транспортному рівні).</t>
+          <t>HTTP (HyperText Transfer Protocol) є протоколом прикладного рівня (Application Layer, Layer 7 моделі OSI). Він визначає семантику запитів і відповідей між клієнтом і сервером, тоді як транспортуванням цих даних займаються протоколи нижчих рівнів, такі як TCP або UDP.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Що означає характеристика 'stateless' (без збереження стану) стосовно протоколу HTTP?</t>
+          <t>Що означає характеристика HTTP 'stateless' (без збереження стану)?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -533,75 +535,95 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Кожен HTTP-запит є незалежним; сервер не зобов'язаний пам'ятати історію попередніх запитів від клієнта.</t>
+          <t>Сервер автоматично розриває TCP-з'єднання відразу після отримання запиту.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Протокол не дозволяє передавати файли та зображення, а лише звичайний текст.</t>
+          <t>Кожен HTTP-запит є незалежним; сервер не зберігає історію чи контекст попередніх запитів у межах самого протоколу.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Клієнт зобов'язаний постійно тримати TCP-з'єднання відкритим.</t>
+          <t>Клієнт не може надсилати більше одного запиту на хвилину.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Сервер ніколи не повертає статус-коди помилок.</t>
+          <t>Протокол HTTP не підтримує передачу зашифрованих даних (HTTPS).</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>30</v>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>HTTP є stateless-протоколом. Це означає, що сервер обробляє кожен запит окремо і ізольовано. Він не зберігає автоматично інформацію про попередні запити того самого клієнта. Для збереження стану на практиці використовуються сторонні механізми (наприклад, Cookies або сесії).</t>
+          <t>HTTP є stateless (без збереження стану) протоколом. Це означає, що кожен запит обробляється як повністю незалежна транзакція, і сервер не пам'ятає попередніх взаємодій з цим клієнтом. Для збереження стану на рівні додатків використовують додаткові механізми, такі як Cookies або сесії.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Хто є первинним автором протоколу HTTP та винахідником концепції World Wide Web (WWW) у CERN у 1991 році? Вкажіть ім'я та прізвище українською мовою.</t>
+          <t>Яка главна відмінність між URL та URN?</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fill-in-the-Blank</t>
+          <t>Multiple Choice</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Тім Бернерс-Лі</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+          <t>URL ідентифікує ресурс і вказує спосіб його отримання (місцезнаходження), тоді як URN лише ідентифікує ресурс за унікальним ім'ям без прив'язки до локації.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>URL використовується тільки для веб-сайтів, а URN — тільки для файлів на локальному диску.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>URN є застарілою версією URL і більше не підтримується сучасними браузерами.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>URL обов'язково містить порт, а URN — ні.</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="n">
-        <v>30</v>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Тім Бернерс-Лі (Tim Berners-Lee) у 1991 році, працюючи в CERN (Європейська організація з ядерних досліджень), розробив перші версії мови HTML, протоколу HTTP та технології URL, що поклало початок всесвітній павутині World Wide Web.</t>
+          <t>URL (Uniform Resource Locator) визначає шлях до ресурсу та спосіб доступу до нього (наприклад, https://example.com/file.html). URN (Uniform Resource Name) визначає унікальне ім'я ресурсу в певному просторі імен незалежно від його розташування (наприклад, urn:isbn:978-3-16-148410-0). Обидва є підмножинами URI.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Яка частина вказаного URL-шляху `https://api.example.com:443/v1/users?role=admin#profile` визначає використовувану схему (протокол)?</t>
+          <t>Яка частина наступного URL-адресу ніколи не надсилається клієнтом (наприклад, браузером) на сервер у складі HTTP-запиту: 'https://example.com/api/users?role=admin#profile'?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -611,177 +633,197 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https</t>
+          <t>role=admin (Query string)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>api.example.com</t>
+          <t>/api/users (Path)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>443</t>
+          <t>#profile (Fragment)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>v1/users</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>role=admin</t>
-        </is>
-      </c>
+          <t>https (Scheme)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>30</v>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Перша частина URL перед двокрапкою з похилими рисками (`https`) називається схемою (Scheme) або протоколом і визначає, який саме стандарт використовуватиметься для доступу до ресурсу.</t>
+          <t>Фрагмент URL (частина після символу #, у цьому випадку #profile) використовується виключно клієнтом (наприклад, браузером для прокручування сторінки до потрібного ID або для SPA-роутингу). Він ніколи не надсилається на сервер у стартовому рядку HTTP-запиту.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Які компоненти входять до складу структури URL-адреси згідно зі специфікацією RFC 3986? Виберіть усі правильні варіанти:</t>
+          <t>Яка основна мета URL-кодування (URL Encoding/Percent-Encoding)?</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Multiple Choice</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Схема (Scheme / протокол)</t>
+          <t>Стиснення URL для зменшення трафіку.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Хост (Host / доменне ім'я або IP-адреса)</t>
+          <t>Безпечне шифрування URL, щоб приховати параметри від зловмисників.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Шлях до ресурсу (Path)</t>
+          <t>Перетворення спеціальних, кириличних або небезпечних символів у безпечний для передачі ASCII-формат з використанням знаку % та шістнадцяткових кодів.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Рядок запиту (Query String / параметри)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Назва операційної системи клієнта</t>
-        </is>
-      </c>
+          <t>Автоматичний переклад URL на англійську мову.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1,2,3,4</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>45</v>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>URL-адреса складається зі схеми (напр. `https`), хоста (напр. `example.com`), порту, ієрархічного шляху до ресурсу (Path), рядка запиту (Query String після `?`) та фрагмента (після `#`). Дані про операційну систему клієнта до складу URL не входять (вони передаються в HTTP-заголовку User-Agent).</t>
+          <t>URL може містити лише обмежений набір символів ASCII. Всі інші символи (пробіли, кирилиця, спецсимволи на кшталт &amp; або =, якщо вони є частиною значення параметра) мають бути закодовані (наприклад, пробіл перетворюється на %20), щоб не порушувати структуру URL.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Який стандартний порт транспортного протоколу TCP використовується за замовчуванням для захищеного з'єднання HTTPS? Вкажіть лише число.</t>
+          <t>Яку роль відіграє обов'язковий порожній рядок (CRLF) в анатомії HTTP-повідомлення?</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fill-in-the-Blank</t>
+          <t>Multiple Choice</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>443</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+          <t>Він вказує на версію протоколу HTTP.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Він відокремлює стартовий рядок (Request/Status Line) від HTTP-заголовків.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Він відокремлює блок HTTP-заголовків від тіла повідомлення (Body).</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Він повідомляє серверу про завершення TCP-з'єднання.</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="n">
-        <v>30</v>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Для стандартного незахищеного з'єднання HTTP за замовчуванням використовується порт 80, а для захищеного шифрованого з'єднання HTTPS — порт 443.</t>
+          <t>В анатомії як HTTP-запиту, так і HTTP-відповіді, порожній рядок (дві послідовності CRLF: \r\n\r\n) є чітким роздільником між метаданими (заголовками) та власне корисним навантаженням (тілом повідомлення). Якщо тіло відсутнє, запит/відповідь завершується цим порожнім рядком.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Який компонент є обов'язковим роздільником між заголовками HTTP-повідомлення та його тілом (якщо воно присутнє)?</t>
+          <t>Які з HTTP-методів згідно зі специфікацією є ІДЕМПОТЕНТНИМИ? (Оберіть усі правильні варіанти)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Multiple Choice</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Один порожній рядок (двосимвольний маркер CRLF)</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Символ крапки з комою</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Кілька знаків дефісу `---`</t>
+          <t>PUT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>HTML-тег `&lt;body&gt;`</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>30</v>
+          <t>1,3,4</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Згідно з RFC 7230, для того щоб сервер або клієнт міг правильно зрозуміти, де закінчуються метадані (заголовки) і починаються байти корисного навантаження (тіло), заголовки обов'язково відокремлюються від тіла одним порожнім рядком (символами переведення каретки та нового рядка - CRLF).</t>
+          <t>Ідемпотентність означає, що виконання одного й того самого запиту кілька разів поспіль дає той самий результат, що й одноразовий виклик. GET (лише зчитує), PUT (повністю заміщує ресурс конкретним вмістом) та DELETE (видаляє ресурс; повторне видалення вже видаленого ресурсу все одно призводить до того, що його немає) є ідемпотентними. POST (створює новий ресурс щоразу) та PATCH (може робити відносні зміни, наприклад, інкремент) не є ідемпотентними.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Який HTTP-запит клієнта зазвичай містить тіло повідомлення (Request Body)?</t>
+          <t>Яка ключова різниця між HTTP-методами POST та PUT при створенні/оновленні ресурсів у REST API?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -791,95 +833,95 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>POST-запит для створення нової сутності на сервері</t>
+          <t>POST надсилає дані у заголовках, а PUT — у тілі запиту.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>GET-запит для отримання вебсторінки</t>
+          <t>PUT є ідемпотентним і зазвичай використовується для створення чи повного оновлення ресурсу за відомим URL (де ID визначає клієнт), тоді як POST не є ідемпотентним і використовується, коли ID ресурсу генерує сервер.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>HEAD-запит для отримання лише метаданих файлу</t>
+          <t>POST використовується лише для оновлення, а PUT — виключно для створення нових записів.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>OPTIONS-запит для перевірки дозволених серверних методів</t>
+          <t>PUT працює лише через HTTPS, а POST — через HTTP та HTTPS.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>30</v>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Запити отримання інформації (GET, HEAD) за специфікацією не повинні містити тіло. Запити типу POST, PUT та PATCH призначені для надсилання даних на сервер (наприклад, JSON або даних форми), тому вони містять тіло повідомлення (Request Body).</t>
+          <t>PUT є ідемпотентним: якщо клієнт знає точний URL ресурсу (наприклад, /users/42) і надсилає PUT-запит, він повністю перезаписує ресурс. Повторні PUT-запити не створять нових користувачів. POST не є ідемпотентним: він надсилається на колекцію (/users), і кожен новий виклик буде створювати новий ресурс із новим ID, згенерованим сервером.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Які HTTP-методи вважаються 'безпечними' (Safe), тобто такими, що не змінюють стан сервера (здійснюють лише читання)? Виберіть усі правильні варіанти:</t>
+          <t>Чим метод PATCH відрізняється від методу PUT?</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Multiple Choice</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH використовується для видалення ресурсів, а PUT — для створення.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>HEAD</t>
+          <t>PUT призначений для часткового оновлення ресурсу (тільки вказаних полів), тоді як PATCH повністю замінює весь ресурс.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OPTIONS</t>
+          <t>PATCH призначений для часткового оновлення ресурсу (передаються лише змінені поля), тоді як PUT вимагає відправки всього представлення ресурсу для його повної заміни.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>DELETE</t>
-        </is>
-      </c>
+          <t>Між ними немає різниці, це синоніми у специфікації HTTP.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1,2,3</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>30</v>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Безпечними методами є ті, що не призводять до зміни стану бази даних чи ресурсів на сервері. Це GET (читання ресурсу), HEAD (читання заголовків без тіла) та OPTIONS (запит параметрів з'єднання). POST та DELETE змінюють стан сервера (створюють чи видаляють сутності), тому вони не є безпечними.</t>
+          <t>Згідно з RFC, метод PUT замінює весь ресурс новим представленням (якщо якісь поля не надіслати, вони можуть бути стерті або скинуті до дефолтних). PATCH (RFC 5789) здійснює часткове оновлення (partial update) — клієнт надсилає лише ті поля, які реально змінилися.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>У чому полягає основне призначення HTTP-методу GET?</t>
+          <t>Який клас статус-кодів HTTP відповідає за помилки, що виникли на стороні КЛІЄНТА (наприклад, неправильний запит, відсутність авторизації тощо)?</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -889,44 +931,46 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Для безпечного читання та отримання представлення конкретного ресурсу чи списку ресурсів.</t>
+          <t>2xx (наприклад, 200, 201)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Для повного оновлення або заміни існуючого ресурсу новими даними.</t>
+          <t>3xx (наприклад, 301, 302)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Для повного видалення ресурсу з бази даних сервера.</t>
+          <t>4xx (наприклад, 400, 404)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Для створення нових записів на сервері.</t>
+          <t>5xx (наприклад, 500, 503)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>30</v>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Метод GET призначений виключно для отримання (читання) інформації з сервера. Він не повинен містити тіло запиту та не має змінювати стан даних на сервері.</t>
+          <t>Коди сімейства 4xx (400 Bad Request, 401 Unauthorized, 403 Forbidden, 404 Not Found тощо) вказують на те, що помилка сталася через неправильні дії клієнта (помилка в запиті, відсутність доступу чи відсутність ресурсу). Коди 5xx вказують на помилки сервера.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Який HTTP-заголовок використовується сервером або клієнтом для опису медіа-формату даних, які реально містяться в тілі повідомлення (наприклад, `application/json` або `text/html`)?</t>
+          <t>У чому різниця між статус-кодами 401 Unauthorized та 403 Forbidden?</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -936,44 +980,46 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Content-Type</t>
+          <t>401 означає, що користувач заблокований адміністратором, а 403 — що сервер тимчасово перевантажений.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Accept</t>
+          <t>401 вказує на відсутність або недійсність аутентифікації (користувач не представився), тоді як 403 вказує на відсутність прав доступу (користувач аутентифікований, але не має дозволу на цю дію).</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>User-Agent</t>
+          <t>401 повертається лише при помилках у базі даних, а 403 — при помилках у мережі.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Ці коди є взаємозамінними і означають одне й те саме.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>30</v>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Заголовок `Content-Type` вказує одержувачу повідомлення (клієнту чи серверу), як саме інтерпретувати байти в тілі повідомлення. Наприклад, `Content-Type: text/html` означає, що в тілі передається HTML-сторінка, а `application/json` — дані у форматі JSON.</t>
+          <t>401 Unauthorized (хоча назва перекладається як 'не авторизований', фактично він означає 'не аутентифікований'): клієнт не надав правильних облікових даних. 403 Forbidden: сервер зрозумів, хто робить запит, але у цього користувача немає прав (ролі/дозволів) для виконання цієї операції.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Що означає перша цифра тризначного HTTP статус-коду відповіді сервера?</t>
+          <t>Як клієнт і сервер взаємодіють для умовного кешування за допомогою заголовків ETag та If-None-Match?</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -983,44 +1029,46 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Клас або категорію відповіді (інформаційна, успіх, перенаправлення, помилка клієнта чи сервера)</t>
+          <t>Сервер надсилає весь файл, а клієнт перевіряє його ETag. Якщо він збігається, клієнт видаляє файл.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Кількість секунд, яку клієнт повинен чекати на відповідь</t>
+          <t>Сервер повертає у відповіді унікальний хеш ресурсу у заголовку ETag. При наступному запиті клієнт надсилає цей хеш у заголовку If-None-Match. Якщо ресурс не змінився, сервер відповідає статус-кодом 304 Not Modified без тіла відповіді.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Версію протоколу HTTP, яку підтримує сервер</t>
+          <t>Клієнт генерує ETag на основі часу запиту, а сервер звіряє його зі своєю базою даних.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Кількість байтів у тілі відповіді</t>
+          <t>Ці заголовки використовуються лише для шифрування трафіку і не мають відношення до кешування.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>30</v>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Класи статус-кодів визначаються першою цифрою: 1xx: Інформаційні відповіді; 2xx: Успішні відповіді (Success); 3xx: Перенаправлення (Redirection); 4xx: Помилка клієнта (Client Error); 5xx: Помилка сервера (Server Error).</t>
+          <t>ETag (Entity Tag) — це унікальний маркер версії ресурсу (зазвичай хеш вмісту). Якщо клієнт уже має цей ресурс у кеші, він робить умовний запит з If-None-Match: [хеш]. Якщо на сервері ресурс не змінився, сервер економить трафік і повертає 304 Not Modified без передачі самого тіла документа.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Що повідомляє клієнту найвідоміший HTTP статус-код `404 Not Found`?</t>
+          <t>Чи є методи класу HttpClient у .NET потокобезпечними (thread-safe), і як рекомендується його використовувати у багатопотоковому середовищі?</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1030,44 +1078,46 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Запитаний ресурс не знайдено на сервері (наприклад, неправильний URL-шлях).</t>
+          <t>Ні, HttpClient не є потокобезпечним. Для кожного потоку необхідно створювати власний екземпляр через new HttpClient().</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Запит виконано успішно і повернуто вміст сторінки.</t>
+          <t>Так, методи відправки запитів HttpClient (такі як SendAsync, GetAsync, PostAsync) є потокобезпечними. Рекомендується перевикористовувати один і той самий екземпляр для багатьох запитів у застосунку.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>На сервері сталася критична помилка в коді.</t>
+          <t>Методи є потокобезпечними лише при використанні синхронних методів, яких у HttpClient немає.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Клієнт не пройшов авторизацію для перегляду сторінки.</t>
+          <t>Потокобезпечність гарантується тільки якщо загорнути кожен виклик у блок lock.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>30</v>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Код `404 Not Found` означає, що сервер успішно встановив з'єднання, але не зміг знайти запитаний ресурс за вказаним клієнтом шляхом. Найчастіше це стається через помилки в написанні URL-адреси.</t>
+          <t>Клас HttpClient розроблений для спільного використання. Його методи відправки запитів є потокобезпечними. Більше того, розробникам наполегливо рекомендується використовувати єдиний (або зареєстрований як Singleton) екземпляр HttpClient протягом усього життєвого циклу застосунку, щоб запобігти вичерпанню сокетів (Socket Exhaustion).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Який клас HTTP статус-кодів вказує на те, що помилка виникла саме на стороні сервера (наприклад, критичний виняток у коді чи збій бази даних)?</t>
+          <t>Чи генерує метод HttpClient.GetAsync() виняток (exception), якщо сервер повертає статус-код помилки, наприклад 404 Not Found або 500 Internal Server Error?</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1077,84 +1127,333 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5xx (наприклад, 500 Internal Server Error)</t>
+          <t>Так, будь-який статус-код помилки (4xx або 5xx) одразу викликає генерацію HttpRequestException.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>4xx (наприклад, 400 Bad Request)</t>
+          <t>Ні, HttpClient успішно повертає об'єкт HttpResponseMessage зі статус-кодом помилки. Щоб згенерувати виняток вручну у разі невдачі, потрібно викликати метод response.EnsureSuccessStatusCode().</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3xx (наприклад, 301 Moved Permanently)</t>
+          <t>Так, але виняток генерується лише для помилок сервера (5xx), а помилки клієнта (4xx) ігноруються.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2xx (наприклад, 200 OK)</t>
+          <t>Виняток генерується лише якщо відповідь не містить тіла (Body).</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>30</v>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Клас статус-кодів `5xx` (наприклад, 500, 502, 503) сигналізує про помилки, які виникли на стороні сервера під час спроби обробити синтаксично правильний запит. Коди `4xx` вказують на помилки з боку клієнта (невірний запит чи відсутність доступу).</t>
+          <t>За замовчуванням методи HttpClient (наприклад, GetAsync, PostAsync) не генерують винятки при отриманні HTTP статус-кодів помилок (4xx/5xx). Вони вважають запит успішно виконаним на рівні транспорту. Для перевірки успішності статусу розробник має перевірити response.IsSuccessStatusCode або викликати EnsureSuccessStatusCode(), який викине HttpRequestException у разі неуспішного статусу.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Чим відрізняється поведінка протоколу HTTP/1.1 порівняно з старішим HTTP/1.0 щодо мережевих TCP-з'єднань? Виберіть усі правильні твердження:</t>
+          <t>У чому полягає небезпека створення нового екземпляра класу HttpClient на кожен HTTP-запит у .NET (наприклад, через конструкцію 'using var client = new HttpClient()')?</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Multiple Choice</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>HTTP/1.1 підтримує постійні з'єднання (Keep-Alive) за замовчуванням, дозволяючи відправляти кілька запитів через один TCP-канал.</t>
+          <t>Об'єкт HttpClient займає занадто багато оперативної пам'яті (до 100 МБ на інстанс).</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>В HTTP/1.0 кожний окремий запит вимагав створення нового TCP-з'єднання з нуля.</t>
+          <t>Хоча сам об'єкт звільняється, базовий сокет TCP переходить у стан TIME_WAIT на кілька хвилин, що при високому навантаженні призводить до вичерпання доступних сокетів (Socket Exhaustion).</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>HTTP/1.1 примусово забороняє будь-яке використання заголовків.</t>
+          <t>HttpClient видає виняток InvalidOperationException, якщо його використовувати більше одного разу.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>HTTP/1.0 повністю працював без використання IP-адрес.</t>
+          <t>Кожен новий екземпляр автоматично очищає DNS-кеш операційної системи.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1,2</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>45</v>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>У старій версії HTTP/1.0 після отримання кожної відповіді TCP-з'єднання відразу закривалося, що вимагало значних ресурсів на постійні рукостискання (handshake). У версії HTTP/1.1 з'явилася підтримка Keep-Alive за замовчуванням: з'єднання залишається відкритим, що дозволяє суттєво зекономити час і трафік при завантаженні сторінки з багатьма елементами.</t>
+          <t>HttpClient реалізує IDisposable, але його утилізація через using не закриває сокет негайно. TCP-сокет залишається у стані TIME_WAIT (зазвичай 4 хвилини) для збору запізнілих пакетів. При частому створенні HttpClient система швидко вичерпає ліміт вільних портів (Socket Exhaustion), і нові запити будуть завершуватися помилкою.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Як вирішити проблему оновлення DNS-записів (DNS stale) при тривалому використанні одного екземпляра HttpClient у сучасному .NET (Core 2.1+) без використання IHttpClientFactory?</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Регулярно викликати метод client.DefaultRequestHeaders.Clear().</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Налаштувати властивість PooledConnectionLifetime у SocketsHttpHandler і передати його в конструктор HttpClient. Це обмежить час життя TCP-з'єднань у пулі, змушуючи клієнт періодично перепідключатися та оновлювати DNS.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Жодного способу немає, оновлення DNS працює лише через сторонні бібліотеки.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Викликати статичний метод HttpClient.ClearDnsCache().</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>У .NET Core 2.1+ під капотом HttpClient використовується SocketsHttpHandler. Налаштувавши PooledConnectionLifetime (наприклад, встановивши його в 2 хвилини), ми змушуємо обробник закривати активні TCP-з'єднання після закінчення цього часу та відкривати нові для наступних запитів. Це автоматично оновлює DNS-записи та вирішує проблему DNS stale, не потребуючи використання IHttpClientFactory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Яка різниця між заголовками запиту Host та Origin?</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Host містить IP-адресу клієнта, а Origin — IP-адресу сервера.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Host вказує доменне ім'я та порт сервера, якому призначений запит (обов'язковий для HTTP/1.1), а Origin надсилається браузером при CORS-запитах і містить лише схему, хост та порт сторінки, з якої ініційовано запит (без шляху).</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Host використовується тільки в HTTP/3, а Origin — тільки в HTTP/1.0.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Host визначає операційну систему клієнта, а Origin — країну походження запиту.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Заголовок Host є обов'язковим в HTTP/1.1 і вказує на цільовий сервер (дозволяє віртуальний хостинг на одному IP). Заголовок Origin автоматично додається браузером під час крос-доменних запитів (CORS) чи POST-запитів і містить джерело (схема, домен, порт), звідки запущено JS-код, але без приватних даних на кшталт шляху /path чи query-параметрів.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Для чого використовується заголовок Content-Type, і чим він відрізняється від заголовка Accept?</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Content-Type використовується для кешування, а Accept — для авторизації.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Content-Type вказує медіа-тип даних, які надсилаються в тілі поточного повідомлення, а Accept вказує серверу, які типи контенту клієнт готовий отримати у відповідь.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Content-Type повідомляє версію операційної системи, а Accept — версію браузера.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Ці заголовки виконують абсолютно однакову функцію і є взаємозамінними.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Content-Type описує формат даних у тілі поточного запиту чи відповіді (наприклад, application/json або text/html). Заголовок Accept надсилається клієнтом, щоб повідомити серверу про свої переваги щодо формату відповіді (наприклад: 'я очікую відповідь у форматі JSON: Accept: application/json').</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Яка основна особливість статус-кодів перенаправлення 301 Moved Permanently та 308 Permanent Redirect порівняно з 302 Found та 307 Temporary Redirect?</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Коди 301 та 308 кешуються браузером за замовчуванням і використовуються для постійної зміни URL ресурсу, тоді як 302 та 307 вказують на тимчасове перенаправлення і не повинні кешуватися надовго.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>301 та 308 використовуються тільки для зображень, а 302 та 307 — для HTML-сторінок.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Коди 301 та 308 вимагають ручного підтвердження від користувача, а 302 та 307 виконання автоматично.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Коди 302 та 307 закривають TCP-з'єднання, а 301 та 308 — тримають його відкритим.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Статус-коди 301 та 308 повідомляють клієнту, що ресурс переїхав на новий URL назавжди. Браузери агресивно кешують це перенаправлення, тому наступні запити одразу йдуть на нову адресу без звернення до старого URL. Коди 302 та 307 означають тимчасове переміщення, тому клієнт повинен продовжувати запитувати оригінальний URL при наступних спробах.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Що визначає заголовок Transfer-Encoding: chunked у HTTP-відповіді?</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Що дані стиснуті за допомогою алгоритму Brotli або Gzip.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Що відповідь буде передаватися частинами (шматками) динамічного розміру, оскільки сервер не знає фінального розміру тіла відповіді на момент початку відправки. При цьому заголовок Content-Length не використовується.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Що клієнт повинен розбити свій наступний POST-запит на кілька частин.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Що з'єднання буде розірвано відразу після отримання першого байта даних.</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Якщо сервер генерує велику або динамічну відповідь (наприклад, рендерить велику сторінку або транслює відео), він не може заздалегідь порахувати і надіслати Content-Length. Використання Transfer-Encoding: chunked дозволяє серверу надсилати дані блоками, де кожен блок починається з його розміру в шістнадцятковому форматі, а передача закінчується блоком нульового розміру.</t>
         </is>
       </c>
     </row>

</xml_diff>